<commit_message>
type subtype script fix
</commit_message>
<xml_diff>
--- a/src/test/resources/TestCoverageDashboard_QA.xlsx
+++ b/src/test/resources/TestCoverageDashboard_QA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\57901\smart-test-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2B0BF4-F9A7-400B-8F68-D85C6A0E3E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F99EDB-2C30-4BDD-AF16-39FB360AD3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79FC711E-34A0-4D45-A805-C86E1CFB22CF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{79FC711E-34A0-4D45-A805-C86E1CFB22CF}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCoverage" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>Functional Area</t>
   </si>
@@ -152,9 +152,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy\ h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="m/d/yyyy h:mm:ss AM/PM"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -306,7 +307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -368,6 +369,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -681,7 +683,7 @@
                   <c:v>Document Management ()</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Validations &amp; Business Rules (25)</c:v>
+                  <c:v>Validations &amp; Business Rules (30)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -702,7 +704,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0.94117647058823528</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1</c:v>
@@ -726,13 +728,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.76</c:v>
+                  <c:v>0.93333333333333335</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -868,7 +870,7 @@
                   <c:v>Document Management ()</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Validations &amp; Business Rules (25)</c:v>
+                  <c:v>Validations &amp; Business Rules (30)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -889,7 +891,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>5.8823529411764705E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -913,13 +915,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.24</c:v>
+                  <c:v>6.6666666666666666E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1055,7 +1057,7 @@
                   <c:v>Document Management ()</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Validations &amp; Business Rules (25)</c:v>
+                  <c:v>Validations &amp; Business Rules (30)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1133,7 +1135,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="bg2"/>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="85000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1242,7 +1246,7 @@
                   <c:v>Document Management ()</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>Validations &amp; Business Rules (25)</c:v>
+                  <c:v>Validations &amp; Business Rules (30)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2405,15 +2409,15 @@
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" customWidth="1"/>
-    <col min="6" max="6" width="8.140625" customWidth="1"/>
-    <col min="7" max="7" width="7.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="32.5703125"/>
+    <col min="2" max="2" customWidth="true" width="24.0"/>
+    <col min="3" max="3" customWidth="true" width="24.5703125"/>
+    <col min="4" max="4" customWidth="true" width="14.7109375"/>
+    <col min="5" max="5" customWidth="true" width="9.140625"/>
+    <col min="6" max="6" customWidth="true" width="8.140625"/>
+    <col min="7" max="7" customWidth="true" width="7.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.28515625"/>
+    <col min="9" max="9" customWidth="true" width="24.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2421,8 +2425,8 @@
         <v>28</v>
       </c>
       <c r="B1" s="23"/>
-      <c r="C1" s="24">
-        <v>46098.618946759256</v>
+      <c r="C1" s="27" t="n">
+        <v>46105.66914611111</v>
       </c>
       <c r="D1" s="25"/>
       <c r="E1" s="23"/>
@@ -2460,58 +2464,58 @@
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="9">
-        <v>25</v>
-      </c>
-      <c r="C3" s="9">
-        <v>19</v>
-      </c>
-      <c r="D3" s="9">
-        <v>6</v>
-      </c>
-      <c r="E3" s="9">
-        <v>0</v>
-      </c>
-      <c r="F3" s="7">
+      <c r="B3" s="9" t="n">
+        <v>30.0</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>28.0</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="7" t="n">
         <f>IF(B3=0,"",C3/B3)</f>
-        <v>0.76</v>
-      </c>
-      <c r="G3" s="7">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="G3" s="7" t="n">
         <f>IFERROR(D3/B3,0)</f>
-        <v>0.24</v>
-      </c>
-      <c r="H3" s="7">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="H3" s="7" t="n">
         <f>IFERROR(E3/B3,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="10">
-        <v>3</v>
-      </c>
-      <c r="C4" s="10">
-        <v>3</v>
-      </c>
-      <c r="D4" s="10">
-        <v>0</v>
-      </c>
-      <c r="E4" s="10">
-        <v>0</v>
-      </c>
-      <c r="F4" s="7">
+      <c r="B4" s="10" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="7" t="n">
         <f t="shared" ref="F4:F16" si="0">IF(B4=0,"",C4/B4)</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G4" s="7" t="n">
         <f t="shared" ref="G4:G14" si="1">IFERROR(D4/B4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H4" s="7" t="n">
         <f t="shared" ref="H4:H14" si="2">IFERROR(E4/B4,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -2526,129 +2530,129 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H5" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H5" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="10">
-        <v>7</v>
-      </c>
-      <c r="C6" s="10">
-        <v>7</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0</v>
-      </c>
-      <c r="E6" s="10">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7">
+      <c r="B6" s="10" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G6" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H6" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="9">
-        <v>17</v>
-      </c>
-      <c r="C7" s="9">
-        <v>17</v>
-      </c>
-      <c r="D7" s="9">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9">
-        <v>0</v>
-      </c>
-      <c r="F7" s="7">
+      <c r="B7" s="9" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G7" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G7" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H7" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="9">
-        <v>1</v>
-      </c>
-      <c r="C8" s="10">
-        <v>1</v>
-      </c>
-      <c r="D8" s="10">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7">
+      <c r="B8" s="9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G8" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H8" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="9">
-        <v>8</v>
-      </c>
-      <c r="C9" s="9">
-        <v>8</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0</v>
-      </c>
-      <c r="E9" s="9">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7">
+      <c r="B9" s="9" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G9" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G9" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -2664,13 +2668,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H10" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -2686,13 +2690,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H11" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -2708,13 +2712,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I12" s="2"/>
     </row>
@@ -2730,13 +2734,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H13" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I13" s="2"/>
     </row>
@@ -2752,13 +2756,13 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="7" t="n">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H14" s="7" t="n">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="I14" s="2"/>
     </row>
@@ -2766,29 +2770,29 @@
       <c r="A15" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="9">
-        <v>10</v>
-      </c>
-      <c r="C15" s="9">
-        <v>10</v>
-      </c>
-      <c r="D15" s="9">
-        <v>0</v>
-      </c>
-      <c r="E15" s="9">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
+      <c r="B15" s="9" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G15" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <f>IFERROR(D15/B15,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <f t="shared" ref="H15:H17" si="3">IFERROR(E15/B15,0)</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -2803,46 +2807,46 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="7" t="n">
         <f>IFERROR(D16/B16,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H16" s="7" t="n">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="15" t="n">
         <f>SUM(B3:B16)</f>
-        <v>71</v>
-      </c>
-      <c r="C17" s="15">
+        <v>76.0</v>
+      </c>
+      <c r="C17" s="15" t="n">
         <f>SUM(C3:C15)</f>
-        <v>65</v>
-      </c>
-      <c r="D17" s="15">
+        <v>74.0</v>
+      </c>
+      <c r="D17" s="15" t="n">
         <f>SUM(D3:D15)</f>
-        <v>6</v>
-      </c>
-      <c r="E17" s="15">
+        <v>2.0</v>
+      </c>
+      <c r="E17" s="15" t="n">
         <f>SUM(E3:E15)</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="16">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="16" t="n">
         <f t="shared" ref="F17" si="4">IFERROR(C17/B17,0)</f>
-        <v>0.91549295774647887</v>
-      </c>
-      <c r="G17" s="16">
+        <v>0.9736842105263158</v>
+      </c>
+      <c r="G17" s="16" t="n">
         <f t="shared" ref="G17" si="5">IFERROR(D17/B17,0)</f>
-        <v>8.4507042253521125E-2</v>
-      </c>
-      <c r="H17" s="16">
+        <v>0.02631578947368421</v>
+      </c>
+      <c r="H17" s="16" t="n">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>
@@ -2887,12 +2891,12 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="14.7109375"/>
+    <col min="2" max="2" customWidth="true" width="23.5703125"/>
+    <col min="5" max="5" customWidth="true" width="18.0"/>
+    <col min="6" max="6" customWidth="true" width="25.7109375"/>
+    <col min="7" max="7" customWidth="true" width="15.140625"/>
+    <col min="8" max="8" customWidth="true" width="10.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30.75" x14ac:dyDescent="0.55000000000000004">
@@ -2919,9 +2923,9 @@
       <c r="E2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="5" t="n">
         <f>TestCoverage!C1</f>
-        <v>46098.618946759256</v>
+        <v>46105.66914611111</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -2938,9 +2942,9 @@
       <c r="E3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="18">
+      <c r="F3" s="18" t="n">
         <f>TestCoverage!B17</f>
-        <v>71</v>
+        <v>76.0</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -2957,9 +2961,9 @@
       <c r="E4" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="18" t="n">
         <f>TestCoverage!C17</f>
-        <v>65</v>
+        <v>74.0</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -2976,9 +2980,9 @@
       <c r="E5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="18" t="n">
         <f>TestCoverage!D17</f>
-        <v>6</v>
+        <v>2.0</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -2995,9 +2999,9 @@
       <c r="E6" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="18" t="n">
         <f>TestCoverage!E17</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
@@ -3014,9 +3018,9 @@
       <c r="E7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="17" t="n">
         <f>IFERROR(F4/F3,"")</f>
-        <v>0.91549295774647887</v>
+        <v>0.9736842105263158</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -3068,11 +3072,11 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="4" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="26.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="37.85546875"/>
+    <col min="2" max="2" customWidth="true" width="14.0"/>
+    <col min="4" max="5" customWidth="true" width="13.85546875"/>
+    <col min="6" max="6" customWidth="true" width="10.42578125"/>
+    <col min="7" max="7" customWidth="true" width="26.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -3103,29 +3107,29 @@
         <f>TestCoverage!A4 &amp; " (" &amp; TestCoverage!B4 &amp; ")"</f>
         <v>RAI Management (3)</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="21" t="n">
         <f>TestCoverage!F4</f>
-        <v>1</v>
-      </c>
-      <c r="C2" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C2" s="21" t="n">
         <f>TestCoverage!G4</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D2" s="21" t="n">
         <f>TestCoverage!H4</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="21">
-        <f>C2 + D2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="21" t="n">
+        <f t="shared" ref="E2:E15" si="0">C2 + D2</f>
+        <v>0.0</v>
+      </c>
+      <c r="F2" s="20" t="n">
         <f>TestCoverage!B4</f>
-        <v>3</v>
-      </c>
-      <c r="G2" s="19">
-        <f>IF($F2=0,1,0)</f>
-        <v>0</v>
+        <v>3.0</v>
+      </c>
+      <c r="G2" s="19" t="n">
+        <f t="shared" ref="G2:G15" si="1">IF($F2=0,1,0)</f>
+        <v>0.0</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3137,25 +3141,25 @@
         <f>TestCoverage!F5</f>
         <v/>
       </c>
-      <c r="C3" s="21">
+      <c r="C3" s="21" t="n">
         <f>TestCoverage!G5</f>
-        <v>0</v>
-      </c>
-      <c r="D3" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D3" s="21" t="n">
         <f>TestCoverage!H5</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="21">
-        <f>C3 + D3</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="20" t="n">
         <f>TestCoverage!B5</f>
-        <v>0</v>
-      </c>
-      <c r="G3" s="19">
-        <f>IF($F3=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G3" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3163,29 +3167,29 @@
         <f>TestCoverage!A6 &amp; " (" &amp; TestCoverage!B6 &amp; ")"</f>
         <v>Workflow &amp; Status Transitions (7)</v>
       </c>
-      <c r="B4" s="21">
+      <c r="B4" s="21" t="n">
         <f>TestCoverage!F6</f>
-        <v>1</v>
-      </c>
-      <c r="C4" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C4" s="21" t="n">
         <f>TestCoverage!G6</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D4" s="21" t="n">
         <f>TestCoverage!H6</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="21">
-        <f>C4 + D4</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="20" t="n">
         <f>TestCoverage!B6</f>
-        <v>7</v>
-      </c>
-      <c r="G4" s="19">
-        <f>IF($F4=0,1,0)</f>
-        <v>0</v>
+        <v>7.0</v>
+      </c>
+      <c r="G4" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3193,29 +3197,29 @@
         <f>TestCoverage!A7 &amp; " (" &amp; TestCoverage!B7 &amp; ")"</f>
         <v>Record Lifecycle Management (17)</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="21" t="n">
         <f>TestCoverage!F7</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C5" s="21" t="n">
         <f>TestCoverage!G7</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D5" s="21" t="n">
         <f>TestCoverage!H7</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="21">
-        <f>C5 + D5</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="20" t="n">
         <f>TestCoverage!B7</f>
-        <v>17</v>
-      </c>
-      <c r="G5" s="19">
-        <f>IF($F5=0,1,0)</f>
-        <v>0</v>
+        <v>17.0</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3223,29 +3227,29 @@
         <f>TestCoverage!A8 &amp; " (" &amp; TestCoverage!B8 &amp; ")"</f>
         <v>User Access &amp; Permissions (1)</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="21" t="n">
         <f>TestCoverage!F8</f>
-        <v>1</v>
-      </c>
-      <c r="C6" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C6" s="21" t="n">
         <f>TestCoverage!G8</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D6" s="21" t="n">
         <f>TestCoverage!H8</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="21">
-        <f>C6 + D6</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="20" t="n">
         <f>TestCoverage!B8</f>
-        <v>1</v>
-      </c>
-      <c r="G6" s="19">
-        <f>IF($F6=0,1,0)</f>
-        <v>0</v>
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3253,29 +3257,29 @@
         <f>TestCoverage!A9 &amp; " (" &amp; TestCoverage!B9 &amp; ")"</f>
         <v>Assignment &amp; Routing (8)</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="21" t="n">
         <f>TestCoverage!F9</f>
-        <v>1</v>
-      </c>
-      <c r="C7" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C7" s="21" t="n">
         <f>TestCoverage!G9</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D7" s="21" t="n">
         <f>TestCoverage!H9</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="21">
-        <f>C7 + D7</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="20" t="n">
         <f>TestCoverage!B9</f>
-        <v>8</v>
-      </c>
-      <c r="G7" s="19">
-        <f>IF($F7=0,1,0)</f>
-        <v>0</v>
+        <v>8.0</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3287,25 +3291,25 @@
         <f>TestCoverage!F10</f>
         <v/>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="21" t="n">
         <f>TestCoverage!G10</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="21" t="n">
         <f>TestCoverage!H10</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="21">
-        <f>C8 + D8</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="20" t="n">
         <f>TestCoverage!B10</f>
-        <v>0</v>
-      </c>
-      <c r="G8" s="19">
-        <f>IF($F8=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3317,25 +3321,25 @@
         <f>TestCoverage!F11</f>
         <v/>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="21" t="n">
         <f>TestCoverage!G11</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="21" t="n">
         <f>TestCoverage!H11</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="21">
-        <f>C9 + D9</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="20" t="n">
         <f>TestCoverage!B11</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="19">
-        <f>IF($F9=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3347,25 +3351,25 @@
         <f>TestCoverage!F12</f>
         <v/>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="21" t="n">
         <f>TestCoverage!G12</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="21" t="n">
         <f>TestCoverage!H12</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="21">
-        <f>C10 + D10</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F10" s="20" t="n">
         <f>TestCoverage!B12</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="19">
-        <f>IF($F10=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3377,25 +3381,25 @@
         <f>TestCoverage!F13</f>
         <v/>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="21" t="n">
         <f>TestCoverage!G13</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="21" t="n">
         <f>TestCoverage!H13</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="21">
-        <f>C11 + D11</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F11" s="20" t="n">
         <f>TestCoverage!B13</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="19">
-        <f>IF($F11=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3407,25 +3411,25 @@
         <f>TestCoverage!F14</f>
         <v/>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="21" t="n">
         <f>TestCoverage!G14</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="21" t="n">
         <f>TestCoverage!H14</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="21">
-        <f>C12 + D12</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F12" s="20" t="n">
         <f>TestCoverage!B14</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="19">
-        <f>IF($F12=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3433,29 +3437,29 @@
         <f>TestCoverage!A15 &amp; " (" &amp; TestCoverage!B15 &amp; ")"</f>
         <v>Timeline &amp; SLA Management (10)</v>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="21" t="n">
         <f>TestCoverage!F15</f>
-        <v>1</v>
-      </c>
-      <c r="C13" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="C13" s="21" t="n">
         <f>TestCoverage!G15</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="21" t="n">
         <f>TestCoverage!H15</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="21">
-        <f>C13 + D13</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="20" t="n">
         <f>TestCoverage!B15</f>
-        <v>10</v>
-      </c>
-      <c r="G13" s="19">
-        <f>IF($F13=0,1,0)</f>
-        <v>0</v>
+        <v>10.0</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -3467,82 +3471,82 @@
         <f>TestCoverage!F16</f>
         <v/>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="21" t="n">
         <f>TestCoverage!G16</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="21">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="21" t="n">
         <f>TestCoverage!H16</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="21">
-        <f>C14 + D14</f>
-        <v>0</v>
-      </c>
-      <c r="F14" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E14" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="20" t="n">
         <f>TestCoverage!B16</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="19">
-        <f>IF($F14=0,1,0)</f>
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="str">
         <f>TestCoverage!A3 &amp; " (" &amp; TestCoverage!B3 &amp; ")"</f>
-        <v>Validations &amp; Business Rules (25)</v>
-      </c>
-      <c r="B15" s="21">
+        <v>Validations &amp; Business Rules (30)</v>
+      </c>
+      <c r="B15" s="21" t="n">
         <f>TestCoverage!F3</f>
-        <v>0.76</v>
-      </c>
-      <c r="C15" s="21">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="C15" s="21" t="n">
         <f>TestCoverage!G3</f>
-        <v>0.24</v>
-      </c>
-      <c r="D15" s="21">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="D15" s="21" t="n">
         <f>TestCoverage!H3</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="21">
-        <f>C15 + D15</f>
-        <v>0.24</v>
-      </c>
-      <c r="F15" s="20">
+        <v>0.0</v>
+      </c>
+      <c r="E15" s="21" t="n">
+        <f t="shared" si="0"/>
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="F15" s="20" t="n">
         <f>TestCoverage!B3</f>
-        <v>25</v>
-      </c>
-      <c r="G15" s="19">
-        <f>IF($F15=0,1,0)</f>
-        <v>0</v>
+        <v>30.0</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <f t="shared" si="1"/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="str">
         <f>TestCoverage!A17 &amp; " (" &amp; TestCoverage!B17 &amp; ")"</f>
-        <v>TOTAL (71)</v>
-      </c>
-      <c r="B16" s="21">
+        <v>TOTAL (76)</v>
+      </c>
+      <c r="B16" s="21" t="n">
         <f>TestCoverage!F17</f>
-        <v>0.91549295774647887</v>
-      </c>
-      <c r="C16" s="21">
+        <v>0.9736842105263158</v>
+      </c>
+      <c r="C16" s="21" t="n">
         <f>TestCoverage!G17</f>
-        <v>8.4507042253521125E-2</v>
-      </c>
-      <c r="D16" s="21">
+        <v>0.02631578947368421</v>
+      </c>
+      <c r="D16" s="21" t="n">
         <f>TestCoverage!H17</f>
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="E16" s="21"/>
-      <c r="F16" s="20">
+      <c r="F16" s="20" t="n">
         <f>TestCoverage!B17</f>
-        <v>71</v>
-      </c>
-      <c r="G16" s="19">
+        <v>76.0</v>
+      </c>
+      <c r="G16" s="19" t="n">
         <f>COUNTIF(F2:F14,0)/COUNTA(A2:A14)</f>
-        <v>0.53846153846153844</v>
+        <v>0.5384615384615384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>